<commit_message>
Add new Excel parameter file for 5-minute intervals
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand2.xlsx
+++ b/inputData/LTM_demand2.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,36 +413,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>group</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>origin</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>destination</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>time</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>number_of_passengers</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>stopover_allowed</t>
         </is>
@@ -471,10 +459,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -491,7 +479,7 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -505,19 +493,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -528,13 +516,13 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -545,19 +533,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +553,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -585,19 +573,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -605,16 +593,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -625,16 +613,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -651,13 +639,13 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -665,13 +653,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -688,16 +676,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="E13" t="n">
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -708,16 +696,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -725,19 +713,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -745,19 +733,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -771,10 +759,10 @@
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>1</v>
@@ -785,13 +773,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E18" t="n">
         <v>2</v>
@@ -805,19 +793,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -825,16 +813,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -848,10 +836,10 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="E21" t="n">
         <v>3</v>
@@ -865,19 +853,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -885,13 +873,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="E23" t="n">
         <v>1</v>
@@ -905,19 +893,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -925,19 +913,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C25" t="n">
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -951,13 +939,13 @@
         <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="E26" t="n">
         <v>2</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -965,16 +953,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C27" t="n">
         <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>1</v>
@@ -991,10 +979,10 @@
         <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>1</v>
@@ -1005,16 +993,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C29" t="n">
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -1025,19 +1013,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1048,16 +1036,16 @@
         <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>143</v>
+        <v>122</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1065,19 +1053,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C32" t="n">
         <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>145</v>
+        <v>122</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1088,13 +1076,13 @@
         <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>158</v>
+        <v>126</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
@@ -1105,16 +1093,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -1125,19 +1113,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C35" t="n">
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1145,16 +1133,16 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="E36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
@@ -1171,10 +1159,10 @@
         <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>161</v>
+        <v>129</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
@@ -1185,16 +1173,16 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>166</v>
+        <v>130</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
         <v>1</v>
@@ -1205,19 +1193,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>167</v>
+        <v>135</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1225,16 +1213,16 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>1</v>
@@ -1245,19 +1233,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>175</v>
+        <v>141</v>
       </c>
       <c r="E41" t="n">
         <v>3</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -1265,19 +1253,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D42" t="n">
-        <v>178</v>
+        <v>141</v>
       </c>
       <c r="E42" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -1285,19 +1273,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>184</v>
+        <v>146</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1311,10 +1299,10 @@
         <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>185</v>
+        <v>154</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -1325,16 +1313,16 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C45" t="n">
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>190</v>
+        <v>154</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>1</v>
@@ -1345,19 +1333,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>204</v>
+        <v>156</v>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1365,16 +1353,16 @@
         <v>46</v>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>221</v>
+        <v>171</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -1388,16 +1376,16 @@
         <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>247</v>
+        <v>183</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -1405,16 +1393,16 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>249</v>
+        <v>212</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -1425,16 +1413,16 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>313</v>
+        <v>367</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>1</v>
@@ -1451,13 +1439,13 @@
         <v>4</v>
       </c>
       <c r="D51" t="n">
-        <v>320</v>
+        <v>396</v>
       </c>
       <c r="E51" t="n">
         <v>2</v>
       </c>
       <c r="F51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1465,19 +1453,19 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
-        <v>334</v>
+        <v>396</v>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1491,13 +1479,13 @@
         <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>345</v>
+        <v>410</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1505,16 +1493,16 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>360</v>
+        <v>413</v>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -1525,16 +1513,16 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>362</v>
+        <v>415</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F55" t="n">
         <v>1</v>
@@ -1545,16 +1533,16 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C56" t="n">
         <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>409</v>
+        <v>419</v>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>1</v>
@@ -1565,19 +1553,19 @@
         <v>56</v>
       </c>
       <c r="B57" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C57" t="n">
         <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>413</v>
+        <v>424</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -1591,10 +1579,10 @@
         <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>437</v>
+        <v>454</v>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
@@ -1611,10 +1599,10 @@
         <v>4</v>
       </c>
       <c r="D59" t="n">
-        <v>441</v>
+        <v>457</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -1628,16 +1616,16 @@
         <v>1</v>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D60" t="n">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="E60" t="n">
         <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -1645,13 +1633,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D61" t="n">
-        <v>468</v>
+        <v>463</v>
       </c>
       <c r="E61" t="n">
         <v>2</v>
@@ -1665,19 +1653,19 @@
         <v>61</v>
       </c>
       <c r="B62" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D62" t="n">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="E62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -1685,19 +1673,19 @@
         <v>62</v>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D63" t="n">
-        <v>484</v>
+        <v>471</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -1705,16 +1693,16 @@
         <v>63</v>
       </c>
       <c r="B64" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C64" t="n">
         <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>498</v>
+        <v>473</v>
       </c>
       <c r="E64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
@@ -1725,19 +1713,19 @@
         <v>64</v>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>506</v>
+        <v>475</v>
       </c>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -1751,13 +1739,13 @@
         <v>2</v>
       </c>
       <c r="D66" t="n">
-        <v>514</v>
+        <v>490</v>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -1765,19 +1753,19 @@
         <v>66</v>
       </c>
       <c r="B67" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D67" t="n">
-        <v>516</v>
+        <v>492</v>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -1785,19 +1773,19 @@
         <v>67</v>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D68" t="n">
-        <v>519</v>
+        <v>495</v>
       </c>
       <c r="E68" t="n">
         <v>4</v>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -1805,19 +1793,19 @@
         <v>68</v>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>525</v>
+        <v>497</v>
       </c>
       <c r="E69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -1828,13 +1816,13 @@
         <v>1</v>
       </c>
       <c r="C70" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D70" t="n">
-        <v>533</v>
+        <v>500</v>
       </c>
       <c r="E70" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
@@ -1845,13 +1833,13 @@
         <v>70</v>
       </c>
       <c r="B71" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D71" t="n">
-        <v>538</v>
+        <v>509</v>
       </c>
       <c r="E71" t="n">
         <v>4</v>
@@ -1865,19 +1853,19 @@
         <v>71</v>
       </c>
       <c r="B72" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>543</v>
+        <v>513</v>
       </c>
       <c r="E72" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -1885,19 +1873,19 @@
         <v>72</v>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>547</v>
+        <v>515</v>
       </c>
       <c r="E73" t="n">
         <v>4</v>
       </c>
       <c r="F73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -1905,16 +1893,16 @@
         <v>73</v>
       </c>
       <c r="B74" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D74" t="n">
-        <v>552</v>
+        <v>515</v>
       </c>
       <c r="E74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74" t="n">
         <v>1</v>
@@ -1925,16 +1913,16 @@
         <v>74</v>
       </c>
       <c r="B75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D75" t="n">
-        <v>558</v>
+        <v>537</v>
       </c>
       <c r="E75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
@@ -1945,16 +1933,16 @@
         <v>75</v>
       </c>
       <c r="B76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C76" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>559</v>
+        <v>539</v>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
@@ -1965,16 +1953,16 @@
         <v>76</v>
       </c>
       <c r="B77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D77" t="n">
-        <v>562</v>
+        <v>548</v>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F77" t="n">
         <v>1</v>
@@ -1991,13 +1979,13 @@
         <v>2</v>
       </c>
       <c r="D78" t="n">
-        <v>566</v>
+        <v>550</v>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -2005,16 +1993,16 @@
         <v>78</v>
       </c>
       <c r="B79" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C79" t="n">
         <v>1</v>
       </c>
       <c r="D79" t="n">
-        <v>576</v>
+        <v>553</v>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F79" t="n">
         <v>0</v>
@@ -2028,16 +2016,16 @@
         <v>1</v>
       </c>
       <c r="C80" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D80" t="n">
-        <v>582</v>
+        <v>556</v>
       </c>
       <c r="E80" t="n">
         <v>1</v>
       </c>
       <c r="F80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -2051,10 +2039,10 @@
         <v>1</v>
       </c>
       <c r="D81" t="n">
-        <v>591</v>
+        <v>561</v>
       </c>
       <c r="E81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F81" t="n">
         <v>0</v>
@@ -2068,13 +2056,13 @@
         <v>1</v>
       </c>
       <c r="C82" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D82" t="n">
-        <v>591</v>
+        <v>568</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
@@ -2085,19 +2073,19 @@
         <v>82</v>
       </c>
       <c r="B83" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D83" t="n">
-        <v>591</v>
+        <v>569</v>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -2105,16 +2093,16 @@
         <v>83</v>
       </c>
       <c r="B84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D84" t="n">
-        <v>592</v>
+        <v>575</v>
       </c>
       <c r="E84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -2131,10 +2119,10 @@
         <v>4</v>
       </c>
       <c r="D85" t="n">
-        <v>592</v>
+        <v>577</v>
       </c>
       <c r="E85" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
@@ -2148,13 +2136,13 @@
         <v>1</v>
       </c>
       <c r="C86" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D86" t="n">
-        <v>604</v>
+        <v>579</v>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F86" t="n">
         <v>1</v>
@@ -2165,16 +2153,16 @@
         <v>86</v>
       </c>
       <c r="B87" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C87" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D87" t="n">
-        <v>606</v>
+        <v>587</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>0</v>
@@ -2188,16 +2176,16 @@
         <v>1</v>
       </c>
       <c r="C88" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D88" t="n">
-        <v>612</v>
+        <v>589</v>
       </c>
       <c r="E88" t="n">
         <v>2</v>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -2205,19 +2193,19 @@
         <v>88</v>
       </c>
       <c r="B89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C89" t="n">
         <v>3</v>
       </c>
       <c r="D89" t="n">
-        <v>624</v>
+        <v>599</v>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -2225,19 +2213,19 @@
         <v>89</v>
       </c>
       <c r="B90" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C90" t="n">
         <v>1</v>
       </c>
       <c r="D90" t="n">
-        <v>629</v>
+        <v>603</v>
       </c>
       <c r="E90" t="n">
         <v>4</v>
       </c>
       <c r="F90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -2245,16 +2233,16 @@
         <v>90</v>
       </c>
       <c r="B91" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D91" t="n">
-        <v>634</v>
+        <v>603</v>
       </c>
       <c r="E91" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -2265,16 +2253,16 @@
         <v>91</v>
       </c>
       <c r="B92" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D92" t="n">
-        <v>641</v>
+        <v>608</v>
       </c>
       <c r="E92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -2285,13 +2273,13 @@
         <v>92</v>
       </c>
       <c r="B93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D93" t="n">
-        <v>646</v>
+        <v>612</v>
       </c>
       <c r="E93" t="n">
         <v>4</v>
@@ -2305,19 +2293,19 @@
         <v>93</v>
       </c>
       <c r="B94" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D94" t="n">
-        <v>646</v>
+        <v>614</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -2328,16 +2316,16 @@
         <v>1</v>
       </c>
       <c r="C95" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D95" t="n">
-        <v>651</v>
+        <v>617</v>
       </c>
       <c r="E95" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -2345,16 +2333,16 @@
         <v>95</v>
       </c>
       <c r="B96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D96" t="n">
-        <v>655</v>
+        <v>633</v>
       </c>
       <c r="E96" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F96" t="n">
         <v>0</v>
@@ -2365,19 +2353,19 @@
         <v>96</v>
       </c>
       <c r="B97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D97" t="n">
-        <v>656</v>
+        <v>636</v>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -2385,16 +2373,16 @@
         <v>97</v>
       </c>
       <c r="B98" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D98" t="n">
-        <v>658</v>
+        <v>640</v>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" t="n">
         <v>1</v>
@@ -2411,7 +2399,7 @@
         <v>1</v>
       </c>
       <c r="D99" t="n">
-        <v>660</v>
+        <v>642</v>
       </c>
       <c r="E99" t="n">
         <v>3</v>
@@ -2425,16 +2413,16 @@
         <v>99</v>
       </c>
       <c r="B100" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C100" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D100" t="n">
-        <v>665</v>
+        <v>643</v>
       </c>
       <c r="E100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F100" t="n">
         <v>1</v>
@@ -2445,19 +2433,19 @@
         <v>100</v>
       </c>
       <c r="B101" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C101" t="n">
         <v>1</v>
       </c>
       <c r="D101" t="n">
-        <v>696</v>
+        <v>658</v>
       </c>
       <c r="E101" t="n">
         <v>4</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -2471,13 +2459,13 @@
         <v>4</v>
       </c>
       <c r="D102" t="n">
-        <v>698</v>
+        <v>661</v>
       </c>
       <c r="E102" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -2485,16 +2473,16 @@
         <v>102</v>
       </c>
       <c r="B103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C103" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D103" t="n">
-        <v>700</v>
+        <v>662</v>
       </c>
       <c r="E103" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F103" t="n">
         <v>1</v>
@@ -2508,13 +2496,13 @@
         <v>1</v>
       </c>
       <c r="C104" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D104" t="n">
-        <v>711</v>
+        <v>674</v>
       </c>
       <c r="E104" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
@@ -2525,19 +2513,19 @@
         <v>104</v>
       </c>
       <c r="B105" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C105" t="n">
         <v>1</v>
       </c>
       <c r="D105" t="n">
-        <v>714</v>
+        <v>679</v>
       </c>
       <c r="E105" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -2545,13 +2533,13 @@
         <v>105</v>
       </c>
       <c r="B106" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D106" t="n">
-        <v>732</v>
+        <v>687</v>
       </c>
       <c r="E106" t="n">
         <v>2</v>
@@ -2565,19 +2553,19 @@
         <v>106</v>
       </c>
       <c r="B107" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D107" t="n">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="E107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -2585,39 +2573,19 @@
         <v>107</v>
       </c>
       <c r="B108" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C108" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D108" t="n">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="E108" t="n">
         <v>1</v>
       </c>
       <c r="F108" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>108</v>
-      </c>
-      <c r="B109" t="n">
-        <v>4</v>
-      </c>
-      <c r="C109" t="n">
-        <v>1</v>
-      </c>
-      <c r="D109" t="n">
-        <v>759</v>
-      </c>
-      <c r="E109" t="n">
-        <v>3</v>
-      </c>
-      <c r="F109" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>